<commit_message>
Sitne izmjene u shemama i prežičene str. 125-129. Dodan novi ormar Y BJP12, prve 2 str.
</commit_message>
<xml_diff>
--- a/HE_Senj/oprema_specifikacija/HE Senj - rashlada - specifikacija opreme_FŠ.xlsx
+++ b/HE_Senj/oprema_specifikacija/HE Senj - rashlada - specifikacija opreme_FŠ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\HE_Senj\oprema_specifikacija\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_missing-docid_{43ACBB0E-F446-464A-8737-AAA2B75F6406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{8EBCFC6E-62EA-4CA0-B89E-65713348A131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-2700" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{324E8A42-1211-42FF-BECF-D2BB17870C58}"/>
+    <workbookView xWindow="-38520" yWindow="-4155" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{324E8A42-1211-42FF-BECF-D2BB17870C58}"/>
   </bookViews>
   <sheets>
     <sheet name="Zadaci" sheetId="1" r:id="rId1"/>
@@ -66,14 +66,14 @@
               <from>
                 <xdr:col>7</xdr:col>
                 <xdr:colOff>137160</xdr:colOff>
-                <xdr:row>227</xdr:row>
-                <xdr:rowOff>121920</xdr:rowOff>
+                <xdr:row>201</xdr:row>
+                <xdr:rowOff>167640</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>7</xdr:col>
                 <xdr:colOff>1965960</xdr:colOff>
-                <xdr:row>232</xdr:row>
-                <xdr:rowOff>121920</xdr:rowOff>
+                <xdr:row>206</xdr:row>
+                <xdr:rowOff>167640</xdr:rowOff>
               </to>
             </anchor>
           </commentPr>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="672" uniqueCount="307">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="670" uniqueCount="305">
   <si>
     <t>Br zadatka</t>
   </si>
@@ -480,9 +480,6 @@
     <t>704.911.4-1</t>
   </si>
   <si>
-    <t>2NO modul - kontakti: 2NC; Au/Ag; vijčani priključak</t>
-  </si>
-  <si>
     <t>704.911.3-1</t>
   </si>
   <si>
@@ -982,20 +979,6 @@
     <t>-2K12, -2K13, -K102.1, -K103.1</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">-H1...-H4, -H101, -H102, -H201, -H202, -H301, -H302, -H401...-H403, -H501...-H503, -H601...-H603, -S101, -S103, -S201, -S203, -S301, -S303; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>-H5…-H8, -H404, -H504, -H604, -H701, -H702, -H703, H801, -H802, -S110</t>
-    </r>
-  </si>
-  <si>
     <t>-S31</t>
   </si>
   <si>
@@ -1042,17 +1025,90 @@
     <t>ne postoje -H8, -H404, -H504, -H604</t>
   </si>
   <si>
-    <t>ne postoji -S110</t>
-  </si>
-  <si>
+    <t>-S101...-S103, -S201...-S203, -S301...-S303</t>
+  </si>
+  <si>
+    <t>-V111</t>
+  </si>
+  <si>
+    <t>-E101...-E104</t>
+  </si>
+  <si>
+    <t>-S151...-S154</t>
+  </si>
+  <si>
+    <t>-X500...-X502, -X505, -X550, -X551</t>
+  </si>
+  <si>
+    <t>PK: Ja moram provjeriti naručene količine</t>
+  </si>
+  <si>
+    <t>-F2, -F6...-F13, -F31...-F34, -F36...-F38</t>
+  </si>
+  <si>
+    <t>-F31...-F34, -F36...-F38</t>
+  </si>
+  <si>
+    <t>-F6...-F10, -F13</t>
+  </si>
+  <si>
+    <t>-F101...-F106</t>
+  </si>
+  <si>
+    <t>-F3...-F5</t>
+  </si>
+  <si>
+    <t>-K3.1, -K4.1, -K5.1</t>
+  </si>
+  <si>
+    <t>-K3.1, -K3.2, -K4.1, -K4.2, -K5.1, -K5.2</t>
+  </si>
+  <si>
+    <t>-A121, -A122</t>
+  </si>
+  <si>
+    <t>-2K01...-2K08, -2K11, -2K14...-2K18, -2K21...-2K28, -2K31...-2K38, -2K41...-2K48, -2K51...-2K55</t>
+  </si>
+  <si>
+    <t>-1K101...-1K108, -1K111...-1K118, -1K121...-1K128, -1K131...-1K138, -1K141...-1K148, -1K151...-1K157</t>
+  </si>
+  <si>
+    <t>-1K01...-1K08, -1K11...-1K18, -1K21...-1K24</t>
+  </si>
+  <si>
+    <t>-U151...-U154, -U158...-U160</t>
+  </si>
+  <si>
+    <t>-U155…-U157</t>
+  </si>
+  <si>
+    <t>-S110</t>
+  </si>
+  <si>
+    <t>-X0, -X100</t>
+  </si>
+  <si>
+    <t>količina iz shema je po komadu</t>
+  </si>
+  <si>
+    <t>-X2, -X3, -X103...-X106, -X200+, -X200-, -X201.5, -X201.7, -X202.1...-X202.4, -X202.6...-X202.8, -X231, -X232, -X252...-X254, -X271, -X291, -X292</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">-S101, -S201, -S301, </t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">-S101, -S201, -S301; </t>
+      <t>-S110</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">-H1...-H4, -H101, -H102, -H201, -H202, -H301, -H302, -H401...-H403, -H501...-H503, -H601...-H603, -S101, -S103, -S201, -S203, -S301, -S303, -S110; </t>
     </r>
     <r>
       <rPr>
@@ -1061,80 +1117,11 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>-S110</t>
+      <t>-H5…-H8, -H404, -H504, -H604, -H701, -H702, -H703, H801, -H802</t>
     </r>
   </si>
   <si>
-    <t>-S101...-S103, -S201...-S203, -S301...-S303</t>
-  </si>
-  <si>
-    <t>-V111</t>
-  </si>
-  <si>
-    <t>-E101...-E104</t>
-  </si>
-  <si>
-    <t>-S151...-S154</t>
-  </si>
-  <si>
-    <t>-X500...-X502, -X505, -X550, -X551</t>
-  </si>
-  <si>
-    <t>PK: Ja moram provjeriti naručene količine</t>
-  </si>
-  <si>
-    <t>-F2, -F6...-F13, -F31...-F34, -F36...-F38</t>
-  </si>
-  <si>
-    <t>-F31...-F34, -F36...-F38</t>
-  </si>
-  <si>
-    <t>-F6...-F10, -F13</t>
-  </si>
-  <si>
-    <t>-F101...-F106</t>
-  </si>
-  <si>
-    <t>-F3...-F5</t>
-  </si>
-  <si>
-    <t>-K3.1, -K4.1, -K5.1</t>
-  </si>
-  <si>
-    <t>-K3.1, -K3.2, -K4.1, -K4.2, -K5.1, -K5.2</t>
-  </si>
-  <si>
-    <t>-A121, -A122</t>
-  </si>
-  <si>
-    <t>-2K01...-2K08, -2K11, -2K14...-2K18, -2K21...-2K28, -2K31...-2K38, -2K41...-2K48, -2K51...-2K55</t>
-  </si>
-  <si>
-    <t>-1K101...-1K108, -1K111...-1K118, -1K121...-1K128, -1K131...-1K138, -1K141...-1K148, -1K151...-1K157</t>
-  </si>
-  <si>
-    <t>-1K01...-1K08, -1K11...-1K18, -1K21...-1K24</t>
-  </si>
-  <si>
-    <t>-U151...-U154, -U158...-U160</t>
-  </si>
-  <si>
-    <t>-U155…-U157</t>
-  </si>
-  <si>
-    <t>dodati u -S110</t>
-  </si>
-  <si>
-    <t>-S110</t>
-  </si>
-  <si>
-    <t>-X0, -X100</t>
-  </si>
-  <si>
-    <t>količina iz shema je po komadu</t>
-  </si>
-  <si>
-    <t>-X2, -X3, -X103...-X106, -X200+, -X200-, -X201.5, -X201.7, -X202.1...-X202.4, -X202.6...-X202.8, -X231, -X232, -X252...-X254, -X271, -X291, -X292</t>
+    <t>2NO modul - kontakti: 2NO; Au/Ag; vijčani priključak</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1472,7 @@
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1520,9 +1507,6 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1617,13 +1601,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="16">
     <cellStyle name="20% - Accent2" xfId="10" builtinId="34"/>
@@ -1678,21 +1655,21 @@
         <xdr:from>
           <xdr:col>7</xdr:col>
           <xdr:colOff>137160</xdr:colOff>
-          <xdr:row>227</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
+          <xdr:row>201</xdr:row>
+          <xdr:rowOff>167640</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>7</xdr:col>
           <xdr:colOff>1965960</xdr:colOff>
-          <xdr:row>232</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
+          <xdr:row>206</xdr:row>
+          <xdr:rowOff>167640</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="1025" name="Comment 1" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75DA0292-9E08-63EC-46F5-9848897A51CE}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EBC8DDB-F335-187F-B2AF-BAB47238D4AA}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2182,8 +2159,8 @@
       <c r="J1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="28" t="s">
-        <v>256</v>
+      <c r="K1" s="27" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="28.8">
@@ -2592,8 +2569,8 @@
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="17" t="s">
-        <v>286</v>
+      <c r="A17" s="16" t="s">
+        <v>282</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>33</v>
@@ -2739,8 +2716,8 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="28.8">
-      <c r="A22" s="17" t="s">
-        <v>285</v>
+      <c r="A22" s="16" t="s">
+        <v>281</v>
       </c>
       <c r="B22" s="9" t="s">
         <v>41</v>
@@ -2768,8 +2745,8 @@
         <f t="shared" si="0"/>
         <v>-2</v>
       </c>
-      <c r="K22" s="20" t="s">
-        <v>257</v>
+      <c r="K22" s="19" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="28.8">
@@ -2860,7 +2837,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K25" s="29"/>
+      <c r="K25" s="28"/>
     </row>
     <row r="26" spans="1:11" ht="86.4">
       <c r="A26" s="9" t="s">
@@ -2979,7 +2956,7 @@
       </c>
     </row>
     <row r="30" spans="1:11" ht="28.8">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="16" t="s">
         <v>57</v>
       </c>
       <c r="B30" s="9" t="s">
@@ -3010,7 +2987,7 @@
       </c>
     </row>
     <row r="31" spans="1:11" ht="57.6">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="16" t="s">
         <v>62</v>
       </c>
       <c r="B31" s="9" t="s">
@@ -3041,8 +3018,8 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="86.4">
-      <c r="A32" s="17" t="s">
-        <v>296</v>
+      <c r="A32" s="16" t="s">
+        <v>292</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>65</v>
@@ -3103,14 +3080,14 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="100.8">
-      <c r="A34" s="47" t="s">
-        <v>260</v>
+      <c r="A34" s="46" t="s">
+        <v>259</v>
       </c>
       <c r="B34" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>258</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>259</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>52</v>
@@ -3186,7 +3163,7 @@
       </c>
     </row>
     <row r="37" spans="1:11" ht="43.2">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="16" t="s">
         <v>57</v>
       </c>
       <c r="B37" s="9" t="s">
@@ -3368,8 +3345,8 @@
       </c>
     </row>
     <row r="43" spans="1:11" ht="28.8">
-      <c r="A43" s="17" t="s">
-        <v>301</v>
+      <c r="A43" s="16" t="s">
+        <v>297</v>
       </c>
       <c r="B43" s="9" t="s">
         <v>90</v>
@@ -3399,8 +3376,8 @@
       </c>
     </row>
     <row r="44" spans="1:11" ht="43.2">
-      <c r="A44" s="17" t="s">
-        <v>300</v>
+      <c r="A44" s="16" t="s">
+        <v>296</v>
       </c>
       <c r="B44" s="9" t="s">
         <v>92</v>
@@ -3431,7 +3408,7 @@
         <v>-2</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="43.2">
@@ -3462,8 +3439,8 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="43.2">
-      <c r="A46" s="17" t="s">
-        <v>299</v>
+      <c r="A46" s="16" t="s">
+        <v>295</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>96</v>
@@ -3492,7 +3469,7 @@
         <v>21</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="57.6">
@@ -3523,8 +3500,8 @@
       </c>
     </row>
     <row r="48" spans="1:11" ht="43.2">
-      <c r="A48" s="17" t="s">
-        <v>297</v>
+      <c r="A48" s="16" t="s">
+        <v>293</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>98</v>
@@ -3553,7 +3530,7 @@
         <v>-3</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="28.8">
@@ -3587,12 +3564,12 @@
         <v>0</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="43.2">
-      <c r="A50" s="17" t="s">
-        <v>298</v>
+      <c r="A50" s="16" t="s">
+        <v>294</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>103</v>
@@ -3621,7 +3598,7 @@
         <v>-17</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="43.2">
@@ -3679,8 +3656,8 @@
       </c>
     </row>
     <row r="53" spans="1:11" ht="43.2">
-      <c r="A53" s="17" t="s">
-        <v>306</v>
+      <c r="A53" s="16" t="s">
+        <v>301</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>106</v>
@@ -3700,8 +3677,8 @@
       <c r="G53" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H53" s="54" t="s">
-        <v>305</v>
+      <c r="H53" s="9" t="s">
+        <v>300</v>
       </c>
       <c r="I53" s="11">
         <v>409</v>
@@ -3710,7 +3687,6 @@
         <f t="shared" si="1"/>
         <v>-403</v>
       </c>
-      <c r="K53" s="53"/>
     </row>
     <row r="54" spans="1:11" ht="28.8">
       <c r="A54" s="9"/>
@@ -3848,8 +3824,8 @@
       </c>
     </row>
     <row r="59" spans="1:11" ht="28.8">
-      <c r="A59" s="17" t="s">
-        <v>304</v>
+      <c r="A59" s="16" t="s">
+        <v>299</v>
       </c>
       <c r="B59" s="9" t="s">
         <v>112</v>
@@ -3869,8 +3845,8 @@
       <c r="G59" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H59" s="54" t="s">
-        <v>305</v>
+      <c r="H59" s="9" t="s">
+        <v>300</v>
       </c>
       <c r="I59" s="11">
         <v>12</v>
@@ -3935,8 +3911,8 @@
       </c>
     </row>
     <row r="62" spans="1:11" ht="43.2">
-      <c r="A62" s="17" t="s">
-        <v>284</v>
+      <c r="A62" s="16" t="s">
+        <v>280</v>
       </c>
       <c r="B62" s="9" t="s">
         <v>115</v>
@@ -3964,11 +3940,11 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K62" s="19"/>
+      <c r="K62" s="18"/>
     </row>
     <row r="63" spans="1:11" ht="72">
-      <c r="A63" s="17" t="s">
-        <v>274</v>
+      <c r="A63" s="16" t="s">
+        <v>303</v>
       </c>
       <c r="B63" s="9" t="s">
         <v>117</v>
@@ -3998,8 +3974,8 @@
       </c>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" s="17" t="s">
-        <v>283</v>
+      <c r="A64" s="16" t="s">
+        <v>279</v>
       </c>
       <c r="B64" s="9" t="s">
         <v>120</v>
@@ -4029,8 +4005,8 @@
       </c>
     </row>
     <row r="65" spans="1:11">
-      <c r="A65" s="17" t="s">
-        <v>275</v>
+      <c r="A65" s="16" t="s">
+        <v>273</v>
       </c>
       <c r="B65" s="9" t="s">
         <v>122</v>
@@ -4060,14 +4036,14 @@
       </c>
     </row>
     <row r="66" spans="1:11">
-      <c r="A66" s="17" t="s">
-        <v>303</v>
+      <c r="A66" s="46" t="s">
+        <v>298</v>
       </c>
       <c r="B66" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="C66" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C66" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="D66" s="11" t="s">
         <v>119</v>
@@ -4081,9 +4057,7 @@
       <c r="G66" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H66" s="16" t="s">
-        <v>302</v>
-      </c>
+      <c r="H66" s="9"/>
       <c r="I66" s="11"/>
       <c r="J66" s="7" t="str">
         <f t="shared" si="1"/>
@@ -4091,17 +4065,17 @@
       </c>
     </row>
     <row r="67" spans="1:11" ht="28.8">
-      <c r="A67" s="22" t="s">
+      <c r="A67" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B67" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B67" s="22" t="s">
+      <c r="C67" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="C67" s="23" t="s">
+      <c r="D67" s="15" t="s">
         <v>128</v>
-      </c>
-      <c r="D67" s="15" t="s">
-        <v>129</v>
       </c>
       <c r="E67" s="11">
         <v>7</v>
@@ -4120,22 +4094,22 @@
         <f t="shared" ref="J67:J97" si="2">IF(ISBLANK(I67),"",E67-I67)</f>
         <v>0</v>
       </c>
-      <c r="K67" s="19"/>
+      <c r="K67" s="18"/>
     </row>
     <row r="68" spans="1:11" ht="43.8" customHeight="1">
-      <c r="A68" s="37" t="s">
-        <v>276</v>
-      </c>
-      <c r="B68" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="C68" s="35" t="s">
-        <v>255</v>
-      </c>
-      <c r="D68" s="36" t="s">
+      <c r="A68" s="36" t="s">
+        <v>274</v>
+      </c>
+      <c r="B68" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="C68" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="D68" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="E68" s="21">
+      <c r="E68" s="20">
         <v>15</v>
       </c>
       <c r="F68" s="11" t="s">
@@ -4145,7 +4119,7 @@
         <v>17</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="I68" s="11">
         <v>7</v>
@@ -4154,24 +4128,24 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K68" s="30" t="s">
-        <v>263</v>
+      <c r="K68" s="29" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="28.8">
-      <c r="A69" s="45" t="s">
-        <v>278</v>
-      </c>
-      <c r="B69" s="42" t="s">
+      <c r="A69" s="44" t="s">
+        <v>276</v>
+      </c>
+      <c r="B69" s="41" t="s">
+        <v>130</v>
+      </c>
+      <c r="C69" s="42" t="s">
         <v>131</v>
       </c>
-      <c r="C69" s="43" t="s">
-        <v>132</v>
-      </c>
-      <c r="D69" s="44" t="s">
+      <c r="D69" s="43" t="s">
         <v>119</v>
       </c>
-      <c r="E69" s="21">
+      <c r="E69" s="20">
         <v>6</v>
       </c>
       <c r="F69" s="11" t="s">
@@ -4190,19 +4164,19 @@
       </c>
     </row>
     <row r="70" spans="1:11" ht="37.200000000000003" customHeight="1">
-      <c r="A70" s="27" t="s">
-        <v>279</v>
-      </c>
-      <c r="B70" s="24" t="s">
+      <c r="A70" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="B70" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="C70" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="C70" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="D70" s="26" t="s">
+      <c r="D70" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="E70" s="21">
+      <c r="E70" s="20">
         <v>6</v>
       </c>
       <c r="F70" s="11" t="s">
@@ -4212,7 +4186,7 @@
         <v>17</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="I70" s="11">
         <v>3</v>
@@ -4223,19 +4197,19 @@
       </c>
     </row>
     <row r="71" spans="1:11" ht="28.8">
-      <c r="A71" s="39" t="s">
+      <c r="A71" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="B71" s="38" t="s">
         <v>135</v>
       </c>
-      <c r="B71" s="39" t="s">
+      <c r="C71" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="C71" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="D71" s="41" t="s">
+      <c r="D71" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="E71" s="21">
+      <c r="E71" s="20">
         <v>3</v>
       </c>
       <c r="F71" s="11" t="s">
@@ -4254,16 +4228,16 @@
       </c>
     </row>
     <row r="72" spans="1:11" ht="28.8">
-      <c r="A72" s="37" t="s">
-        <v>282</v>
-      </c>
-      <c r="B72" s="34" t="s">
+      <c r="A72" s="36" t="s">
+        <v>302</v>
+      </c>
+      <c r="B72" s="33" t="s">
+        <v>137</v>
+      </c>
+      <c r="C72" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="C72" s="35" t="s">
-        <v>139</v>
-      </c>
-      <c r="D72" s="36" t="s">
+      <c r="D72" s="35" t="s">
         <v>119</v>
       </c>
       <c r="E72" s="11">
@@ -4275,9 +4249,7 @@
       <c r="G72" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H72" s="9" t="s">
-        <v>281</v>
-      </c>
+      <c r="H72" s="9"/>
       <c r="I72" s="11">
         <v>3</v>
       </c>
@@ -4287,16 +4259,16 @@
       </c>
     </row>
     <row r="73" spans="1:11" ht="28.8">
-      <c r="A73" s="42" t="s">
+      <c r="A73" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="B73" s="41" t="s">
         <v>140</v>
       </c>
-      <c r="B73" s="42" t="s">
+      <c r="C73" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="C73" s="43" t="s">
-        <v>142</v>
-      </c>
-      <c r="D73" s="44" t="s">
+      <c r="D73" s="43" t="s">
         <v>119</v>
       </c>
       <c r="E73" s="11">
@@ -4318,16 +4290,16 @@
       </c>
     </row>
     <row r="74" spans="1:11" ht="28.8">
-      <c r="A74" s="24" t="s">
+      <c r="A74" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="B74" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="B74" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="C74" s="25" t="s">
-        <v>268</v>
-      </c>
-      <c r="D74" s="26" t="s">
+      <c r="C74" s="24" t="s">
+        <v>267</v>
+      </c>
+      <c r="D74" s="25" t="s">
         <v>119</v>
       </c>
       <c r="E74" s="11">
@@ -4349,16 +4321,16 @@
       </c>
     </row>
     <row r="75" spans="1:11" ht="28.8">
-      <c r="A75" s="38" t="s">
-        <v>275</v>
-      </c>
-      <c r="B75" s="31" t="s">
+      <c r="A75" s="37" t="s">
+        <v>273</v>
+      </c>
+      <c r="B75" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="C75" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="C75" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="D75" s="33" t="s">
+      <c r="D75" s="32" t="s">
         <v>119</v>
       </c>
       <c r="E75" s="11">
@@ -4380,16 +4352,16 @@
       </c>
     </row>
     <row r="76" spans="1:11">
-      <c r="A76" s="38" t="s">
-        <v>275</v>
-      </c>
-      <c r="B76" s="33" t="s">
+      <c r="A76" s="37" t="s">
+        <v>273</v>
+      </c>
+      <c r="B76" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C76" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="C76" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="D76" s="33" t="s">
+      <c r="D76" s="32" t="s">
         <v>119</v>
       </c>
       <c r="E76" s="11">
@@ -4412,13 +4384,13 @@
     </row>
     <row r="77" spans="1:11" ht="43.2">
       <c r="A77" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B77" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="B77" s="9" t="s">
+      <c r="C77" s="10" t="s">
         <v>150</v>
-      </c>
-      <c r="C77" s="10" t="s">
-        <v>151</v>
       </c>
       <c r="D77" s="11" t="s">
         <v>52</v>
@@ -4442,14 +4414,14 @@
       </c>
     </row>
     <row r="78" spans="1:11" ht="28.8">
-      <c r="A78" s="46" t="s">
-        <v>295</v>
+      <c r="A78" s="45" t="s">
+        <v>291</v>
       </c>
       <c r="B78" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C78" s="10" t="s">
         <v>152</v>
-      </c>
-      <c r="C78" s="10" t="s">
-        <v>153</v>
       </c>
       <c r="D78" s="11" t="s">
         <v>48</v>
@@ -4471,19 +4443,19 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K78" s="19" t="s">
-        <v>264</v>
+      <c r="K78" s="18" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="79" spans="1:11" ht="28.8">
-      <c r="A79" s="46" t="s">
-        <v>294</v>
+      <c r="A79" s="45" t="s">
+        <v>290</v>
       </c>
       <c r="B79" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C79" s="10" t="s">
         <v>154</v>
-      </c>
-      <c r="C79" s="10" t="s">
-        <v>155</v>
       </c>
       <c r="D79" s="11" t="s">
         <v>48</v>
@@ -4505,20 +4477,20 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K79" s="29"/>
+      <c r="K79" s="28"/>
     </row>
     <row r="80" spans="1:11" ht="28.8">
       <c r="A80" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B80" s="9" t="s">
         <v>156</v>
-      </c>
-      <c r="B80" s="9" t="s">
-        <v>157</v>
       </c>
       <c r="C80" s="10">
         <v>943405</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E80" s="11">
         <v>1</v>
@@ -4540,16 +4512,16 @@
     </row>
     <row r="81" spans="1:11" ht="28.8">
       <c r="A81" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B81" s="9" t="s">
         <v>159</v>
-      </c>
-      <c r="B81" s="9" t="s">
-        <v>160</v>
       </c>
       <c r="C81" s="10">
         <v>93444012</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E81" s="11">
         <v>1</v>
@@ -4571,16 +4543,16 @@
     </row>
     <row r="82" spans="1:11">
       <c r="A82" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C82" s="10">
         <v>13094006</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E82" s="11">
         <v>1</v>
@@ -4602,16 +4574,16 @@
     </row>
     <row r="83" spans="1:11">
       <c r="A83" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C83" s="10">
         <v>22944016</v>
       </c>
       <c r="D83" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E83" s="11">
         <v>1</v>
@@ -4633,16 +4605,16 @@
     </row>
     <row r="84" spans="1:11">
       <c r="A84" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C84" s="10">
         <v>13994006</v>
       </c>
       <c r="D84" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E84" s="11">
         <v>1</v>
@@ -4664,16 +4636,16 @@
     </row>
     <row r="85" spans="1:11" ht="28.8">
       <c r="A85" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B85" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C85" s="10">
         <v>13091001</v>
       </c>
       <c r="D85" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E85" s="11">
         <v>1</v>
@@ -4695,13 +4667,13 @@
     </row>
     <row r="86" spans="1:11">
       <c r="A86" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="B86" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="B86" s="9" t="s">
+      <c r="C86" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="C86" s="10" t="s">
-        <v>168</v>
       </c>
       <c r="D86" s="11" t="s">
         <v>48</v>
@@ -4725,14 +4697,14 @@
       </c>
     </row>
     <row r="87" spans="1:11" ht="28.8">
-      <c r="A87" s="17" t="s">
-        <v>289</v>
+      <c r="A87" s="16" t="s">
+        <v>285</v>
       </c>
       <c r="B87" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="C87" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="C87" s="10" t="s">
-        <v>170</v>
       </c>
       <c r="D87" s="11" t="s">
         <v>48</v>
@@ -4756,14 +4728,14 @@
       </c>
     </row>
     <row r="88" spans="1:11" ht="28.8">
-      <c r="A88" s="17" t="s">
-        <v>293</v>
+      <c r="A88" s="16" t="s">
+        <v>289</v>
       </c>
       <c r="B88" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C88" s="10" t="s">
         <v>171</v>
-      </c>
-      <c r="C88" s="10" t="s">
-        <v>172</v>
       </c>
       <c r="D88" s="11" t="s">
         <v>48</v>
@@ -4787,14 +4759,14 @@
       </c>
     </row>
     <row r="89" spans="1:11" ht="43.2">
-      <c r="A89" s="17" t="s">
-        <v>293</v>
+      <c r="A89" s="16" t="s">
+        <v>289</v>
       </c>
       <c r="B89" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="C89" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="C89" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="D89" s="11" t="s">
         <v>48</v>
@@ -4818,14 +4790,14 @@
       </c>
     </row>
     <row r="90" spans="1:11" ht="28.8">
-      <c r="A90" s="17" t="s">
-        <v>291</v>
+      <c r="A90" s="16" t="s">
+        <v>287</v>
       </c>
       <c r="B90" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="C90" s="10" t="s">
         <v>175</v>
-      </c>
-      <c r="C90" s="10" t="s">
-        <v>176</v>
       </c>
       <c r="D90" s="11" t="s">
         <v>48</v>
@@ -4850,13 +4822,13 @@
     </row>
     <row r="91" spans="1:11" ht="28.8">
       <c r="A91" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B91" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="B91" s="9" t="s">
+      <c r="C91" s="10" t="s">
         <v>178</v>
-      </c>
-      <c r="C91" s="10" t="s">
-        <v>179</v>
       </c>
       <c r="D91" s="11" t="s">
         <v>48</v>
@@ -4881,13 +4853,13 @@
     </row>
     <row r="92" spans="1:11" ht="28.8">
       <c r="A92" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B92" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B92" s="9" t="s">
+      <c r="C92" s="10" t="s">
         <v>181</v>
-      </c>
-      <c r="C92" s="10" t="s">
-        <v>182</v>
       </c>
       <c r="D92" s="11" t="s">
         <v>48</v>
@@ -4911,14 +4883,14 @@
       </c>
     </row>
     <row r="93" spans="1:11" ht="28.8">
-      <c r="A93" s="17" t="s">
-        <v>290</v>
+      <c r="A93" s="16" t="s">
+        <v>286</v>
       </c>
       <c r="B93" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="C93" s="10" t="s">
         <v>183</v>
-      </c>
-      <c r="C93" s="10" t="s">
-        <v>184</v>
       </c>
       <c r="D93" s="11" t="s">
         <v>48</v>
@@ -4943,13 +4915,13 @@
     </row>
     <row r="94" spans="1:11" ht="28.8">
       <c r="A94" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B94" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B94" s="9" t="s">
+      <c r="C94" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="C94" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="D94" s="11" t="s">
         <v>48</v>
@@ -4966,18 +4938,18 @@
         <v>-2</v>
       </c>
       <c r="K94" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="28.8">
       <c r="A95" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B95" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B95" s="9" t="s">
+      <c r="C95" s="10" t="s">
         <v>189</v>
-      </c>
-      <c r="C95" s="10" t="s">
-        <v>190</v>
       </c>
       <c r="D95" s="11" t="s">
         <v>48</v>
@@ -5001,14 +4973,14 @@
       </c>
     </row>
     <row r="96" spans="1:11" ht="28.8">
-      <c r="A96" s="17" t="s">
-        <v>292</v>
+      <c r="A96" s="16" t="s">
+        <v>288</v>
       </c>
       <c r="B96" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="C96" s="10" t="s">
         <v>191</v>
-      </c>
-      <c r="C96" s="10" t="s">
-        <v>192</v>
       </c>
       <c r="D96" s="11" t="s">
         <v>48</v>
@@ -5033,13 +5005,13 @@
     </row>
     <row r="97" spans="1:11" ht="28.8">
       <c r="A97" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B97" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="B97" s="9" t="s">
+      <c r="C97" s="10" t="s">
         <v>194</v>
-      </c>
-      <c r="C97" s="10" t="s">
-        <v>195</v>
       </c>
       <c r="D97" s="11" t="s">
         <v>48</v>
@@ -5064,13 +5036,13 @@
     </row>
     <row r="98" spans="1:11" ht="28.8">
       <c r="A98" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B98" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="B98" s="9" t="s">
+      <c r="C98" s="10" t="s">
         <v>197</v>
-      </c>
-      <c r="C98" s="10" t="s">
-        <v>198</v>
       </c>
       <c r="D98" s="11" t="s">
         <v>48</v>
@@ -5095,10 +5067,10 @@
     </row>
     <row r="99" spans="1:11" ht="28.8">
       <c r="A99" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C99" s="10">
         <v>29450</v>
@@ -5123,20 +5095,20 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K99" s="29"/>
+      <c r="K99" s="28"/>
     </row>
     <row r="100" spans="1:11">
       <c r="A100" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="B100" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B100" s="9" t="s">
+      <c r="C100" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="C100" s="10" t="s">
+      <c r="D100" s="11" t="s">
         <v>202</v>
-      </c>
-      <c r="D100" s="11" t="s">
-        <v>203</v>
       </c>
       <c r="E100" s="11">
         <v>2</v>
@@ -5158,16 +5130,16 @@
     </row>
     <row r="101" spans="1:11">
       <c r="A101" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B101" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="C101" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="C101" s="10" t="s">
-        <v>205</v>
-      </c>
       <c r="D101" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E101" s="11">
         <v>1</v>
@@ -5179,27 +5151,27 @@
         <v>17</v>
       </c>
       <c r="H101" s="9"/>
-      <c r="I101" s="55">
+      <c r="I101" s="11">
         <v>1</v>
       </c>
       <c r="J101" s="7">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K101" s="19"/>
+      <c r="K101" s="18"/>
     </row>
     <row r="102" spans="1:11" ht="43.2">
       <c r="A102" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B102" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="B102" s="9" t="s">
+      <c r="C102" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="C102" s="10" t="s">
+      <c r="D102" s="11" t="s">
         <v>208</v>
-      </c>
-      <c r="D102" s="11" t="s">
-        <v>209</v>
       </c>
       <c r="E102" s="11">
         <v>1</v>
@@ -5218,14 +5190,14 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K102" s="20"/>
+      <c r="K102" s="19"/>
     </row>
     <row r="103" spans="1:11" ht="28.8">
       <c r="A103" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B103" s="9" t="s">
         <v>210</v>
-      </c>
-      <c r="B103" s="9" t="s">
-        <v>211</v>
       </c>
       <c r="C103" s="10">
         <v>2864011</v>
@@ -5253,16 +5225,16 @@
     </row>
     <row r="104" spans="1:11" ht="28.8">
       <c r="A104" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B104" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="B104" s="9" t="s">
+      <c r="C104" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="C104" s="10" t="s">
+      <c r="D104" s="11" t="s">
         <v>214</v>
-      </c>
-      <c r="D104" s="11" t="s">
-        <v>215</v>
       </c>
       <c r="E104" s="11">
         <v>2</v>
@@ -5274,7 +5246,7 @@
         <v>93</v>
       </c>
       <c r="H104" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I104" s="11"/>
       <c r="J104" s="7" t="str">
@@ -5282,18 +5254,18 @@
         <v/>
       </c>
       <c r="K104" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="28.8">
-      <c r="A105" s="17" t="s">
-        <v>270</v>
+      <c r="A105" s="16" t="s">
+        <v>269</v>
       </c>
       <c r="B105" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="C105" s="10" t="s">
         <v>217</v>
-      </c>
-      <c r="C105" s="10" t="s">
-        <v>218</v>
       </c>
       <c r="D105" s="11" t="s">
         <v>102</v>
@@ -5308,7 +5280,7 @@
         <v>17</v>
       </c>
       <c r="H105" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I105" s="11">
         <v>2</v>
@@ -5317,17 +5289,17 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="K105" s="19"/>
+      <c r="K105" s="18"/>
     </row>
     <row r="106" spans="1:11" ht="43.2">
-      <c r="A106" s="17" t="s">
-        <v>272</v>
+      <c r="A106" s="16" t="s">
+        <v>271</v>
       </c>
       <c r="B106" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="C106" s="18" t="s">
-        <v>266</v>
+        <v>218</v>
+      </c>
+      <c r="C106" s="17" t="s">
+        <v>265</v>
       </c>
       <c r="D106" s="11" t="s">
         <v>102</v>
@@ -5342,7 +5314,7 @@
         <v>17</v>
       </c>
       <c r="H106" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I106" s="11">
         <v>11</v>
@@ -5353,14 +5325,14 @@
       </c>
     </row>
     <row r="107" spans="1:11" ht="43.2">
-      <c r="A107" s="17" t="s">
-        <v>272</v>
+      <c r="A107" s="16" t="s">
+        <v>271</v>
       </c>
       <c r="B107" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="C107" s="10" t="s">
         <v>220</v>
-      </c>
-      <c r="C107" s="10" t="s">
-        <v>221</v>
       </c>
       <c r="D107" s="11" t="s">
         <v>102</v>
@@ -5385,13 +5357,13 @@
     </row>
     <row r="108" spans="1:11" ht="28.8">
       <c r="A108" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B108" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="C108" s="10" t="s">
         <v>222</v>
-      </c>
-      <c r="C108" s="10" t="s">
-        <v>223</v>
       </c>
       <c r="D108" s="11" t="s">
         <v>102</v>
@@ -5413,17 +5385,17 @@
         <f t="shared" si="3"/>
         <v>-1</v>
       </c>
-      <c r="K108" s="19"/>
+      <c r="K108" s="18"/>
     </row>
     <row r="109" spans="1:11">
-      <c r="A109" s="17" t="s">
-        <v>273</v>
+      <c r="A109" s="16" t="s">
+        <v>272</v>
       </c>
       <c r="B109" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="C109" s="10" t="s">
         <v>224</v>
-      </c>
-      <c r="C109" s="10" t="s">
-        <v>225</v>
       </c>
       <c r="D109" s="11" t="s">
         <v>102</v>
@@ -5445,20 +5417,20 @@
         <f t="shared" si="3"/>
         <v>-1</v>
       </c>
-      <c r="K109" s="19"/>
+      <c r="K109" s="18"/>
     </row>
     <row r="110" spans="1:11" ht="43.2">
       <c r="A110" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="B110" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="B110" s="9" t="s">
+      <c r="C110" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="C110" s="10" t="s">
+      <c r="D110" s="11" t="s">
         <v>228</v>
-      </c>
-      <c r="D110" s="11" t="s">
-        <v>229</v>
       </c>
       <c r="E110" s="11">
         <v>1</v>
@@ -5479,17 +5451,17 @@
       </c>
     </row>
     <row r="111" spans="1:11" ht="57.6">
-      <c r="A111" s="17" t="s">
-        <v>287</v>
+      <c r="A111" s="16" t="s">
+        <v>283</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C111" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D111" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E111" s="11">
         <v>5</v>
@@ -5508,22 +5480,22 @@
         <f t="shared" si="3"/>
         <v>-2</v>
       </c>
-      <c r="K111" s="20" t="s">
-        <v>288</v>
+      <c r="K111" s="19" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="72">
       <c r="A112" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B112" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B112" s="9" t="s">
+      <c r="C112" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="C112" s="10" t="s">
-        <v>233</v>
-      </c>
       <c r="D112" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E112" s="11">
         <v>2</v>
@@ -5558,10 +5530,10 @@
     <row r="114" spans="1:10" ht="43.2">
       <c r="A114" s="9"/>
       <c r="B114" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="C114" s="10" t="s">
         <v>234</v>
-      </c>
-      <c r="C114" s="10" t="s">
-        <v>235</v>
       </c>
       <c r="D114" s="11" t="s">
         <v>15</v>
@@ -5584,13 +5556,13 @@
     </row>
     <row r="115" spans="1:10" ht="28.8">
       <c r="A115" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="B115" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="B115" s="9" t="s">
+      <c r="C115" s="10" t="s">
         <v>237</v>
-      </c>
-      <c r="C115" s="10" t="s">
-        <v>238</v>
       </c>
       <c r="D115" s="11" t="s">
         <v>15</v>
@@ -5640,13 +5612,13 @@
     </row>
     <row r="117" spans="1:10">
       <c r="A117" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B117" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="B117" s="9" t="s">
+      <c r="C117" s="14" t="s">
         <v>240</v>
-      </c>
-      <c r="C117" s="14" t="s">
-        <v>241</v>
       </c>
       <c r="D117" s="11" t="s">
         <v>15</v>
@@ -5661,7 +5633,7 @@
         <v>93</v>
       </c>
       <c r="H117" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I117" s="11"/>
       <c r="J117" s="7" t="str">
@@ -5674,10 +5646,10 @@
         <v>36</v>
       </c>
       <c r="B118" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="C118" s="14" t="s">
         <v>243</v>
-      </c>
-      <c r="C118" s="14" t="s">
-        <v>244</v>
       </c>
       <c r="D118" s="11" t="s">
         <v>15</v>
@@ -5692,7 +5664,7 @@
         <v>93</v>
       </c>
       <c r="H118" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I118" s="11"/>
       <c r="J118" s="7" t="str">
@@ -5705,10 +5677,10 @@
         <v>43</v>
       </c>
       <c r="B119" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="C119" s="10" t="s">
         <v>245</v>
-      </c>
-      <c r="C119" s="10" t="s">
-        <v>246</v>
       </c>
       <c r="D119" s="11" t="s">
         <v>15</v>
@@ -5723,7 +5695,7 @@
         <v>93</v>
       </c>
       <c r="H119" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I119" s="11"/>
       <c r="J119" s="7" t="str">
@@ -5733,13 +5705,13 @@
     </row>
     <row r="120" spans="1:10">
       <c r="A120" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B120" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="B120" s="9" t="s">
+      <c r="C120" s="10" t="s">
         <v>248</v>
-      </c>
-      <c r="C120" s="10" t="s">
-        <v>249</v>
       </c>
       <c r="D120" s="11" t="s">
         <v>15</v>
@@ -5754,7 +5726,7 @@
         <v>93</v>
       </c>
       <c r="H120" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I120" s="11"/>
       <c r="J120" s="7" t="str">
@@ -5764,13 +5736,13 @@
     </row>
     <row r="121" spans="1:10">
       <c r="A121" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B121" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="B121" s="9" t="s">
+      <c r="C121" s="10" t="s">
         <v>251</v>
-      </c>
-      <c r="C121" s="10" t="s">
-        <v>252</v>
       </c>
       <c r="D121" s="11" t="s">
         <v>15</v>
@@ -5785,7 +5757,7 @@
         <v>93</v>
       </c>
       <c r="H121" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I121" s="11"/>
       <c r="J121" s="7" t="str">
@@ -5805,44 +5777,44 @@
       <c r="I122" s="15"/>
       <c r="J122" s="7"/>
     </row>
-    <row r="123" spans="1:10">
-      <c r="A123" s="49"/>
-      <c r="B123" s="51" t="s">
+    <row r="123" spans="1:10" ht="199.95" customHeight="1">
+      <c r="A123" s="48"/>
+      <c r="B123" s="50" t="s">
+        <v>252</v>
+      </c>
+      <c r="C123" s="49" t="s">
         <v>253</v>
       </c>
-      <c r="C123" s="50" t="s">
-        <v>254</v>
-      </c>
-      <c r="D123" s="48" t="s">
+      <c r="D123" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="E123" s="52">
-        <v>1</v>
-      </c>
-      <c r="F123" s="48" t="s">
+      <c r="E123" s="51">
+        <v>1</v>
+      </c>
+      <c r="F123" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="G123" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="H123" s="49"/>
-      <c r="I123" s="49"/>
-      <c r="J123" s="50" t="str">
+      <c r="G123" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="H123" s="48"/>
+      <c r="I123" s="48"/>
+      <c r="J123" s="49" t="str">
         <f>IF(ISBLANK(I123), "", E123-I123)</f>
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:10">
-      <c r="A124" s="49"/>
-      <c r="B124" s="51"/>
-      <c r="C124" s="50"/>
-      <c r="D124" s="48"/>
-      <c r="E124" s="52"/>
-      <c r="F124" s="48"/>
-      <c r="G124" s="48"/>
-      <c r="H124" s="49"/>
-      <c r="I124" s="49"/>
-      <c r="J124" s="50"/>
+    <row r="124" spans="1:10" ht="199.95" customHeight="1">
+      <c r="A124" s="48"/>
+      <c r="B124" s="50"/>
+      <c r="C124" s="49"/>
+      <c r="D124" s="47"/>
+      <c r="E124" s="51"/>
+      <c r="F124" s="47"/>
+      <c r="G124" s="47"/>
+      <c r="H124" s="48"/>
+      <c r="I124" s="48"/>
+      <c r="J124" s="49"/>
     </row>
   </sheetData>
   <autoFilter ref="B1:F114" xr:uid="{22550ED4-55A0-4F53-98B1-D10F42FD3934}"/>

</xml_diff>

<commit_message>
Senj cut outi na vratima za Y BJP14 CDP01.
</commit_message>
<xml_diff>
--- a/HE_Senj/oprema_specifikacija/HE Senj - rashlada - specifikacija opreme_FŠ.xlsx
+++ b/HE_Senj/oprema_specifikacija/HE Senj - rashlada - specifikacija opreme_FŠ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr showObjects="none" dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\HE_Senj\oprema_specifikacija\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{8EBCFC6E-62EA-4CA0-B89E-65713348A131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{86FCF3D7-A2E1-4982-98B2-2DEBBBACBA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-4155" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{324E8A42-1211-42FF-BECF-D2BB17870C58}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{324E8A42-1211-42FF-BECF-D2BB17870C58}"/>
   </bookViews>
   <sheets>
     <sheet name="Zadaci" sheetId="1" r:id="rId1"/>
@@ -65,15 +65,15 @@
             <anchor>
               <from>
                 <xdr:col>7</xdr:col>
-                <xdr:colOff>137160</xdr:colOff>
+                <xdr:colOff>133350</xdr:colOff>
                 <xdr:row>201</xdr:row>
-                <xdr:rowOff>167640</xdr:rowOff>
+                <xdr:rowOff>171450</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>7</xdr:col>
-                <xdr:colOff>1965960</xdr:colOff>
+                <xdr:colOff>1962150</xdr:colOff>
                 <xdr:row>206</xdr:row>
-                <xdr:rowOff>167640</xdr:rowOff>
+                <xdr:rowOff>171450</xdr:rowOff>
               </to>
             </anchor>
           </commentPr>
@@ -1654,22 +1654,22 @@
       <xdr:twoCellAnchor editAs="absolute">
         <xdr:from>
           <xdr:col>7</xdr:col>
-          <xdr:colOff>137160</xdr:colOff>
+          <xdr:colOff>133350</xdr:colOff>
           <xdr:row>201</xdr:row>
-          <xdr:rowOff>167640</xdr:rowOff>
+          <xdr:rowOff>171450</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>7</xdr:col>
-          <xdr:colOff>1965960</xdr:colOff>
+          <xdr:colOff>1962150</xdr:colOff>
           <xdr:row>206</xdr:row>
-          <xdr:rowOff>167640</xdr:rowOff>
+          <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="1025" name="Comment 1" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EBC8DDB-F335-187F-B2AF-BAB47238D4AA}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{03B79FA2-4A9D-ADC8-49BF-E520E3C941DA}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1679,8 +1679,8 @@
           </xdr:nvSpPr>
           <xdr:spPr bwMode="auto">
             <a:xfrm>
-              <a:off x="13296900" y="68412360"/>
-              <a:ext cx="1828800" cy="914400"/>
+              <a:off x="12934950" y="75352275"/>
+              <a:ext cx="1828800" cy="952500"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -2074,11 +2074,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF9C89D7-F039-449C-80CB-745BA4392DCD}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="121.5546875" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="121.5703125" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2089,7 +2089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="43.2">
+    <row r="2" spans="1:2" ht="45">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2097,7 +2097,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="129.6">
+    <row r="3" spans="1:2" ht="135">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2113,22 +2113,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:xdr="http://purl.oclc.org/ooxml/drawingml/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0791F9D3-C3E8-4198-906E-F1EBBAF01A10}">
   <dimension ref="A1:K124"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="45.21875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="45.28515625" style="1" customWidth="1"/>
     <col min="2" max="2" width="63" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="33" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="38.21875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="38.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" thickBot="1">
+    <row r="1" spans="1:11" ht="30.75" thickBot="1">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -2163,7 +2163,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8">
+    <row r="2" spans="1:11" ht="30">
       <c r="A2" s="6"/>
       <c r="B2" s="6" t="s">
         <v>14</v>
@@ -2186,7 +2186,8 @@
       <c r="H2" s="6"/>
       <c r="I2" s="8"/>
       <c r="J2" s="7" t="str">
-        <f t="shared" ref="J2:J34" si="0">IF(ISBLANK(I2),"",E2-I2)</f>
+        <f>IF(ISBLANK(I2),"",
+IF(F2="set",100*E2-I2,E2-I2))</f>
         <v/>
       </c>
     </row>
@@ -2213,11 +2214,12 @@
       <c r="H3" s="9"/>
       <c r="I3" s="11"/>
       <c r="J3" s="7" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J3:J66" si="0">IF(ISBLANK(I3),"",
+IF(F3="set",100*E3-I3,E3-I3))</f>
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" ht="30">
       <c r="A4" s="9"/>
       <c r="B4" s="9" t="s">
         <v>20</v>
@@ -2271,7 +2273,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="28.8">
+    <row r="6" spans="1:11" ht="30">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
         <v>22</v>
@@ -2433,7 +2435,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="28.8">
+    <row r="12" spans="1:11" ht="30">
       <c r="A12" s="9"/>
       <c r="B12" s="9" t="s">
         <v>28</v>
@@ -2487,7 +2489,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" ht="30">
       <c r="A14" s="9"/>
       <c r="B14" s="9" t="s">
         <v>30</v>
@@ -2541,7 +2543,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="28.8">
+    <row r="16" spans="1:11" ht="30">
       <c r="A16" s="9"/>
       <c r="B16" s="9" t="s">
         <v>32</v>
@@ -2599,7 +2601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="28.8">
+    <row r="18" spans="1:11" ht="30">
       <c r="A18" s="9" t="s">
         <v>34</v>
       </c>
@@ -2661,7 +2663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="28.8">
+    <row r="20" spans="1:11" ht="30">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
         <v>38</v>
@@ -2688,7 +2690,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" ht="30">
       <c r="A21" s="9"/>
       <c r="B21" s="9" t="s">
         <v>39</v>
@@ -2715,7 +2717,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="28.8">
+    <row r="22" spans="1:11" ht="30">
       <c r="A22" s="16" t="s">
         <v>281</v>
       </c>
@@ -2749,7 +2751,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="28.8">
+    <row r="23" spans="1:11" ht="30">
       <c r="A23" s="9"/>
       <c r="B23" s="9" t="s">
         <v>42</v>
@@ -2807,7 +2809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="25.2" customHeight="1">
+    <row r="25" spans="1:11" ht="25.15" customHeight="1">
       <c r="A25" s="9" t="s">
         <v>45</v>
       </c>
@@ -2839,7 +2841,7 @@
       </c>
       <c r="K25" s="28"/>
     </row>
-    <row r="26" spans="1:11" ht="86.4">
+    <row r="26" spans="1:11" ht="105">
       <c r="A26" s="9" t="s">
         <v>49</v>
       </c>
@@ -2870,7 +2872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="72">
+    <row r="27" spans="1:11" ht="75">
       <c r="A27" s="9"/>
       <c r="B27" s="9" t="s">
         <v>53</v>
@@ -2897,7 +2899,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="28.8">
+    <row r="28" spans="1:11" ht="30">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
         <v>55</v>
@@ -2924,7 +2926,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="57.6">
+    <row r="29" spans="1:11" ht="60">
       <c r="A29" s="9" t="s">
         <v>57</v>
       </c>
@@ -2955,7 +2957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="28.8">
+    <row r="30" spans="1:11" ht="30">
       <c r="A30" s="16" t="s">
         <v>57</v>
       </c>
@@ -2986,7 +2988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="57.6">
+    <row r="31" spans="1:11" ht="75">
       <c r="A31" s="16" t="s">
         <v>62</v>
       </c>
@@ -3017,7 +3019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="86.4">
+    <row r="32" spans="1:11" ht="105">
       <c r="A32" s="16" t="s">
         <v>292</v>
       </c>
@@ -3048,7 +3050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="72">
+    <row r="33" spans="1:11" ht="90">
       <c r="A33" s="9" t="s">
         <v>67</v>
       </c>
@@ -3079,7 +3081,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="100.8">
+    <row r="34" spans="1:11" ht="120">
       <c r="A34" s="46" t="s">
         <v>259</v>
       </c>
@@ -3108,7 +3110,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="57.6">
+    <row r="35" spans="1:11" ht="60">
       <c r="A35" s="9"/>
       <c r="B35" s="9" t="s">
         <v>70</v>
@@ -3131,11 +3133,11 @@
       <c r="H35" s="9"/>
       <c r="I35" s="11"/>
       <c r="J35" s="7" t="str">
-        <f t="shared" ref="J35:J66" si="1">IF(ISBLANK(I35),"",E35-I35)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="43.2">
+    <row r="36" spans="1:11" ht="45">
       <c r="A36" s="9"/>
       <c r="B36" s="9" t="s">
         <v>72</v>
@@ -3158,11 +3160,11 @@
       <c r="H36" s="9"/>
       <c r="I36" s="11"/>
       <c r="J36" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="43.2">
+    <row r="37" spans="1:11" ht="45">
       <c r="A37" s="16" t="s">
         <v>57</v>
       </c>
@@ -3189,11 +3191,11 @@
         <v>1</v>
       </c>
       <c r="J37" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="28.8">
+    <row r="38" spans="1:11" ht="45">
       <c r="A38" s="9"/>
       <c r="B38" s="9" t="s">
         <v>76</v>
@@ -3216,11 +3218,11 @@
       <c r="H38" s="9"/>
       <c r="I38" s="11"/>
       <c r="J38" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="57.6">
+    <row r="39" spans="1:11" ht="60">
       <c r="A39" s="9" t="s">
         <v>78</v>
       </c>
@@ -3247,11 +3249,11 @@
         <v>1</v>
       </c>
       <c r="J39" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="28.8">
+    <row r="40" spans="1:11" ht="30">
       <c r="A40" s="9" t="s">
         <v>81</v>
       </c>
@@ -3278,11 +3280,11 @@
         <v>2</v>
       </c>
       <c r="J40" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="28.8">
+    <row r="41" spans="1:11" ht="45">
       <c r="A41" s="9" t="s">
         <v>84</v>
       </c>
@@ -3309,11 +3311,11 @@
         <v>1</v>
       </c>
       <c r="J41" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="43.2">
+    <row r="42" spans="1:11" ht="45">
       <c r="A42" s="9" t="s">
         <v>87</v>
       </c>
@@ -3340,11 +3342,11 @@
         <v>2</v>
       </c>
       <c r="J42" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="28.8">
+    <row r="43" spans="1:11" ht="45">
       <c r="A43" s="16" t="s">
         <v>297</v>
       </c>
@@ -3371,11 +3373,11 @@
         <v>3</v>
       </c>
       <c r="J43" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="43.2">
+    <row r="44" spans="1:11" ht="45">
       <c r="A44" s="16" t="s">
         <v>296</v>
       </c>
@@ -3404,14 +3406,14 @@
         <v>7</v>
       </c>
       <c r="J44" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-2</v>
       </c>
       <c r="K44" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="43.2">
+    <row r="45" spans="1:11" ht="45">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
         <v>95</v>
@@ -3434,11 +3436,11 @@
       <c r="H45" s="9"/>
       <c r="I45" s="11"/>
       <c r="J45" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="43.2">
+    <row r="46" spans="1:11" ht="60">
       <c r="A46" s="16" t="s">
         <v>295</v>
       </c>
@@ -3465,14 +3467,14 @@
         <v>20</v>
       </c>
       <c r="J46" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="K46" s="1" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="57.6">
+    <row r="47" spans="1:11" ht="60">
       <c r="A47" s="9"/>
       <c r="B47" s="9" t="s">
         <v>97</v>
@@ -3495,11 +3497,11 @@
       <c r="H47" s="9"/>
       <c r="I47" s="11"/>
       <c r="J47" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="43.2">
+    <row r="48" spans="1:11" ht="60">
       <c r="A48" s="16" t="s">
         <v>293</v>
       </c>
@@ -3526,14 +3528,14 @@
         <v>43</v>
       </c>
       <c r="J48" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-3</v>
       </c>
       <c r="K48" s="1" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="28.8">
+    <row r="49" spans="1:11" ht="45">
       <c r="A49" s="9" t="s">
         <v>99</v>
       </c>
@@ -3560,14 +3562,14 @@
         <v>2</v>
       </c>
       <c r="J49" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K49" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="43.2">
+    <row r="50" spans="1:11" ht="60">
       <c r="A50" s="16" t="s">
         <v>294</v>
       </c>
@@ -3594,14 +3596,14 @@
         <v>47</v>
       </c>
       <c r="J50" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-17</v>
       </c>
       <c r="K50" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="43.2">
+    <row r="51" spans="1:11" ht="45">
       <c r="A51" s="9"/>
       <c r="B51" s="9" t="s">
         <v>104</v>
@@ -3624,11 +3626,11 @@
       <c r="H51" s="9"/>
       <c r="I51" s="11"/>
       <c r="J51" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="57.6">
+    <row r="52" spans="1:11" ht="60">
       <c r="A52" s="9"/>
       <c r="B52" s="9" t="s">
         <v>105</v>
@@ -3651,11 +3653,11 @@
       <c r="H52" s="9"/>
       <c r="I52" s="11"/>
       <c r="J52" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="43.2">
+    <row r="53" spans="1:11" ht="45">
       <c r="A53" s="16" t="s">
         <v>301</v>
       </c>
@@ -3684,11 +3686,11 @@
         <v>409</v>
       </c>
       <c r="J53" s="7">
-        <f t="shared" si="1"/>
-        <v>-403</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="28.8">
+        <f t="shared" si="0"/>
+        <v>191</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="30">
       <c r="A54" s="9"/>
       <c r="B54" s="9" t="s">
         <v>107</v>
@@ -3711,11 +3713,11 @@
       <c r="H54" s="9"/>
       <c r="I54" s="11"/>
       <c r="J54" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="28.8">
+    <row r="55" spans="1:11" ht="30">
       <c r="A55" s="9"/>
       <c r="B55" s="9" t="s">
         <v>108</v>
@@ -3738,11 +3740,11 @@
       <c r="H55" s="9"/>
       <c r="I55" s="11"/>
       <c r="J55" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="28.8">
+    <row r="56" spans="1:11" ht="45">
       <c r="A56" s="9"/>
       <c r="B56" s="9" t="s">
         <v>109</v>
@@ -3765,11 +3767,11 @@
       <c r="H56" s="9"/>
       <c r="I56" s="11"/>
       <c r="J56" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="28.8">
+    <row r="57" spans="1:11" ht="45">
       <c r="A57" s="9"/>
       <c r="B57" s="9" t="s">
         <v>110</v>
@@ -3792,11 +3794,11 @@
       <c r="H57" s="9"/>
       <c r="I57" s="11"/>
       <c r="J57" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="28.8">
+    <row r="58" spans="1:11" ht="30">
       <c r="A58" s="9"/>
       <c r="B58" s="9" t="s">
         <v>111</v>
@@ -3819,11 +3821,11 @@
       <c r="H58" s="9"/>
       <c r="I58" s="11"/>
       <c r="J58" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="28.8">
+    <row r="59" spans="1:11" ht="30">
       <c r="A59" s="16" t="s">
         <v>299</v>
       </c>
@@ -3852,11 +3854,11 @@
         <v>12</v>
       </c>
       <c r="J59" s="7">
-        <f t="shared" si="1"/>
-        <v>-11</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="28.8">
+        <f t="shared" si="0"/>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="30">
       <c r="A60" s="9"/>
       <c r="B60" s="9" t="s">
         <v>113</v>
@@ -3879,11 +3881,11 @@
       <c r="H60" s="9"/>
       <c r="I60" s="11"/>
       <c r="J60" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="28.8">
+    <row r="61" spans="1:11" ht="30">
       <c r="A61" s="9"/>
       <c r="B61" s="9" t="s">
         <v>114</v>
@@ -3906,11 +3908,11 @@
       <c r="H61" s="9"/>
       <c r="I61" s="11"/>
       <c r="J61" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="43.2">
+    <row r="62" spans="1:11" ht="45">
       <c r="A62" s="16" t="s">
         <v>280</v>
       </c>
@@ -3937,12 +3939,12 @@
         <v>1</v>
       </c>
       <c r="J62" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K62" s="18"/>
     </row>
-    <row r="63" spans="1:11" ht="72">
+    <row r="63" spans="1:11" ht="75">
       <c r="A63" s="16" t="s">
         <v>303</v>
       </c>
@@ -3969,7 +3971,7 @@
         <v>25</v>
       </c>
       <c r="J63" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
     </row>
@@ -4000,7 +4002,7 @@
         <v>9</v>
       </c>
       <c r="J64" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
@@ -4031,7 +4033,7 @@
         <v>1</v>
       </c>
       <c r="J65" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -4060,11 +4062,11 @@
       <c r="H66" s="9"/>
       <c r="I66" s="11"/>
       <c r="J66" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="28.8">
+    <row r="67" spans="1:11" ht="30">
       <c r="A67" s="21" t="s">
         <v>125</v>
       </c>
@@ -4091,12 +4093,13 @@
         <v>7</v>
       </c>
       <c r="J67" s="7">
-        <f t="shared" ref="J67:J97" si="2">IF(ISBLANK(I67),"",E67-I67)</f>
+        <f t="shared" ref="J67:J122" si="1">IF(ISBLANK(I67),"",
+IF(F67="set",100*E67-I67,E67-I67))</f>
         <v>0</v>
       </c>
       <c r="K67" s="18"/>
     </row>
-    <row r="68" spans="1:11" ht="43.8" customHeight="1">
+    <row r="68" spans="1:11" ht="43.9" customHeight="1">
       <c r="A68" s="36" t="s">
         <v>274</v>
       </c>
@@ -4125,14 +4128,14 @@
         <v>7</v>
       </c>
       <c r="J68" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="K68" s="29" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="28.8">
+    <row r="69" spans="1:11" ht="30">
       <c r="A69" s="44" t="s">
         <v>276</v>
       </c>
@@ -4159,11 +4162,11 @@
         <v>6</v>
       </c>
       <c r="J69" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="37.200000000000003" customHeight="1">
+    <row r="70" spans="1:11" ht="37.15" customHeight="1">
       <c r="A70" s="26" t="s">
         <v>277</v>
       </c>
@@ -4192,11 +4195,11 @@
         <v>3</v>
       </c>
       <c r="J70" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="28.8">
+    <row r="71" spans="1:11" ht="30">
       <c r="A71" s="38" t="s">
         <v>134</v>
       </c>
@@ -4223,11 +4226,11 @@
         <v>3</v>
       </c>
       <c r="J71" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="28.8">
+    <row r="72" spans="1:11" ht="30">
       <c r="A72" s="36" t="s">
         <v>302</v>
       </c>
@@ -4254,11 +4257,11 @@
         <v>3</v>
       </c>
       <c r="J72" s="7">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" ht="28.8">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="30">
       <c r="A73" s="41" t="s">
         <v>139</v>
       </c>
@@ -4285,11 +4288,11 @@
         <v>3</v>
       </c>
       <c r="J73" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="28.8">
+    <row r="74" spans="1:11" ht="30">
       <c r="A74" s="23" t="s">
         <v>142</v>
       </c>
@@ -4316,11 +4319,11 @@
         <v>3</v>
       </c>
       <c r="J74" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="28.8">
+    <row r="75" spans="1:11" ht="30">
       <c r="A75" s="37" t="s">
         <v>273</v>
       </c>
@@ -4347,7 +4350,7 @@
         <v>1</v>
       </c>
       <c r="J75" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -4378,11 +4381,11 @@
         <v>1</v>
       </c>
       <c r="J76" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="43.2">
+    <row r="77" spans="1:11" ht="45">
       <c r="A77" s="9" t="s">
         <v>148</v>
       </c>
@@ -4409,11 +4412,11 @@
         <v>1</v>
       </c>
       <c r="J77" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="28.8">
+    <row r="78" spans="1:11" ht="30">
       <c r="A78" s="45" t="s">
         <v>291</v>
       </c>
@@ -4440,14 +4443,14 @@
         <v>6</v>
       </c>
       <c r="J78" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K78" s="18" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="28.8">
+    <row r="79" spans="1:11" ht="30">
       <c r="A79" s="45" t="s">
         <v>290</v>
       </c>
@@ -4474,12 +4477,12 @@
         <v>3</v>
       </c>
       <c r="J79" s="7">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>297</v>
       </c>
       <c r="K79" s="28"/>
     </row>
-    <row r="80" spans="1:11" ht="28.8">
+    <row r="80" spans="1:11" ht="30">
       <c r="A80" s="9" t="s">
         <v>155</v>
       </c>
@@ -4506,11 +4509,11 @@
         <v>1</v>
       </c>
       <c r="J80" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="28.8">
+    <row r="81" spans="1:11" ht="30">
       <c r="A81" s="9" t="s">
         <v>158</v>
       </c>
@@ -4537,7 +4540,7 @@
         <v>1</v>
       </c>
       <c r="J81" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -4568,7 +4571,7 @@
         <v>1</v>
       </c>
       <c r="J82" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -4599,7 +4602,7 @@
         <v>1</v>
       </c>
       <c r="J83" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -4630,11 +4633,11 @@
         <v>1</v>
       </c>
       <c r="J84" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="28.8">
+    <row r="85" spans="1:11" ht="30">
       <c r="A85" s="9" t="s">
         <v>158</v>
       </c>
@@ -4661,7 +4664,7 @@
         <v>1</v>
       </c>
       <c r="J85" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -4692,11 +4695,11 @@
         <v>1</v>
       </c>
       <c r="J86" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="28.8">
+    <row r="87" spans="1:11" ht="30">
       <c r="A87" s="16" t="s">
         <v>285</v>
       </c>
@@ -4723,11 +4726,11 @@
         <v>16</v>
       </c>
       <c r="J87" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="28.8">
+    <row r="88" spans="1:11" ht="30">
       <c r="A88" s="16" t="s">
         <v>289</v>
       </c>
@@ -4754,11 +4757,11 @@
         <v>3</v>
       </c>
       <c r="J88" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="43.2">
+    <row r="89" spans="1:11" ht="45">
       <c r="A89" s="16" t="s">
         <v>289</v>
       </c>
@@ -4785,11 +4788,11 @@
         <v>3</v>
       </c>
       <c r="J89" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="28.8">
+    <row r="90" spans="1:11" ht="30">
       <c r="A90" s="16" t="s">
         <v>287</v>
       </c>
@@ -4816,11 +4819,11 @@
         <v>6</v>
       </c>
       <c r="J90" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="28.8">
+    <row r="91" spans="1:11" ht="30">
       <c r="A91" s="9" t="s">
         <v>176</v>
       </c>
@@ -4847,11 +4850,11 @@
         <v>1</v>
       </c>
       <c r="J91" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="28.8">
+    <row r="92" spans="1:11" ht="30">
       <c r="A92" s="9" t="s">
         <v>179</v>
       </c>
@@ -4878,11 +4881,11 @@
         <v>1</v>
       </c>
       <c r="J92" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="28.8">
+    <row r="93" spans="1:11" ht="30">
       <c r="A93" s="16" t="s">
         <v>286</v>
       </c>
@@ -4909,11 +4912,11 @@
         <v>7</v>
       </c>
       <c r="J93" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="28.8">
+    <row r="94" spans="1:11" ht="30">
       <c r="A94" s="9" t="s">
         <v>184</v>
       </c>
@@ -4934,14 +4937,14 @@
         <v>2</v>
       </c>
       <c r="J94" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-2</v>
       </c>
       <c r="K94" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="28.8">
+    <row r="95" spans="1:11" ht="30">
       <c r="A95" s="9" t="s">
         <v>187</v>
       </c>
@@ -4968,11 +4971,11 @@
         <v>2</v>
       </c>
       <c r="J95" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="28.8">
+    <row r="96" spans="1:11" ht="30">
       <c r="A96" s="16" t="s">
         <v>288</v>
       </c>
@@ -4999,11 +5002,11 @@
         <v>6</v>
       </c>
       <c r="J96" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="1:11" ht="28.8">
+    <row r="97" spans="1:11" ht="30">
       <c r="A97" s="9" t="s">
         <v>192</v>
       </c>
@@ -5030,11 +5033,11 @@
         <v>6</v>
       </c>
       <c r="J97" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:11" ht="28.8">
+    <row r="98" spans="1:11" ht="30">
       <c r="A98" s="9" t="s">
         <v>195</v>
       </c>
@@ -5061,11 +5064,11 @@
         <v>2</v>
       </c>
       <c r="J98" s="7">
-        <f t="shared" ref="J98:J112" si="3">IF(ISBLANK(I98),"",E98-I98)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="28.8">
+    <row r="99" spans="1:11" ht="45">
       <c r="A99" s="9" t="s">
         <v>195</v>
       </c>
@@ -5092,7 +5095,7 @@
         <v>2</v>
       </c>
       <c r="J99" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K99" s="28"/>
@@ -5124,7 +5127,7 @@
         <v>2</v>
       </c>
       <c r="J100" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -5155,12 +5158,12 @@
         <v>1</v>
       </c>
       <c r="J101" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K101" s="18"/>
     </row>
-    <row r="102" spans="1:11" ht="43.2">
+    <row r="102" spans="1:11" ht="45">
       <c r="A102" s="9" t="s">
         <v>205</v>
       </c>
@@ -5187,12 +5190,12 @@
         <v>1</v>
       </c>
       <c r="J102" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K102" s="19"/>
     </row>
-    <row r="103" spans="1:11" ht="28.8">
+    <row r="103" spans="1:11" ht="30">
       <c r="A103" s="9" t="s">
         <v>209</v>
       </c>
@@ -5219,11 +5222,11 @@
         <v>2</v>
       </c>
       <c r="J103" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="28.8">
+    <row r="104" spans="1:11" ht="30">
       <c r="A104" s="9" t="s">
         <v>211</v>
       </c>
@@ -5250,14 +5253,14 @@
       </c>
       <c r="I104" s="11"/>
       <c r="J104" s="7" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K104" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="28.8">
+    <row r="105" spans="1:11" ht="45">
       <c r="A105" s="16" t="s">
         <v>269</v>
       </c>
@@ -5286,12 +5289,12 @@
         <v>2</v>
       </c>
       <c r="J105" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="K105" s="18"/>
     </row>
-    <row r="106" spans="1:11" ht="43.2">
+    <row r="106" spans="1:11" ht="45">
       <c r="A106" s="16" t="s">
         <v>271</v>
       </c>
@@ -5320,11 +5323,11 @@
         <v>11</v>
       </c>
       <c r="J106" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="107" spans="1:11" ht="43.2">
+    <row r="107" spans="1:11" ht="60">
       <c r="A107" s="16" t="s">
         <v>271</v>
       </c>
@@ -5351,11 +5354,11 @@
         <v>11</v>
       </c>
       <c r="J107" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="28.8">
+    <row r="108" spans="1:11" ht="45">
       <c r="A108" s="9" t="s">
         <v>270</v>
       </c>
@@ -5382,7 +5385,7 @@
         <v>7</v>
       </c>
       <c r="J108" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="K108" s="18"/>
@@ -5414,12 +5417,12 @@
         <v>4</v>
       </c>
       <c r="J109" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="K109" s="18"/>
     </row>
-    <row r="110" spans="1:11" ht="43.2">
+    <row r="110" spans="1:11" ht="45">
       <c r="A110" s="9" t="s">
         <v>225</v>
       </c>
@@ -5446,11 +5449,11 @@
         <v>1</v>
       </c>
       <c r="J110" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:11" ht="57.6">
+    <row r="111" spans="1:11" ht="60">
       <c r="A111" s="16" t="s">
         <v>283</v>
       </c>
@@ -5477,14 +5480,14 @@
         <v>7</v>
       </c>
       <c r="J111" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>-2</v>
       </c>
       <c r="K111" s="19" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="72">
+    <row r="112" spans="1:11" ht="90">
       <c r="A112" s="9" t="s">
         <v>230</v>
       </c>
@@ -5511,7 +5514,7 @@
         <v>2</v>
       </c>
       <c r="J112" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -5525,9 +5528,12 @@
       <c r="G113" s="11"/>
       <c r="H113" s="9"/>
       <c r="I113" s="11"/>
-      <c r="J113" s="7"/>
-    </row>
-    <row r="114" spans="1:10" ht="43.2">
+      <c r="J113" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="45">
       <c r="A114" s="9"/>
       <c r="B114" s="9" t="s">
         <v>233</v>
@@ -5550,11 +5556,11 @@
       <c r="H114" s="9"/>
       <c r="I114" s="11"/>
       <c r="J114" s="7" t="str">
-        <f t="shared" ref="J114:J121" si="4">IF(ISBLANK(I114),"",E114-I114)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="28.8">
+    <row r="115" spans="1:10" ht="30">
       <c r="A115" s="9" t="s">
         <v>235</v>
       </c>
@@ -5579,11 +5585,11 @@
       <c r="H115" s="9"/>
       <c r="I115" s="11"/>
       <c r="J115" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="28.8">
+    <row r="116" spans="1:10" ht="30">
       <c r="A116" s="9"/>
       <c r="B116" s="9" t="s">
         <v>106</v>
@@ -5606,7 +5612,7 @@
       <c r="H116" s="9"/>
       <c r="I116" s="11"/>
       <c r="J116" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -5637,7 +5643,7 @@
       </c>
       <c r="I117" s="11"/>
       <c r="J117" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -5668,7 +5674,7 @@
       </c>
       <c r="I118" s="11"/>
       <c r="J118" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -5699,7 +5705,7 @@
       </c>
       <c r="I119" s="11"/>
       <c r="J119" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -5730,7 +5736,7 @@
       </c>
       <c r="I120" s="11"/>
       <c r="J120" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -5761,7 +5767,7 @@
       </c>
       <c r="I121" s="11"/>
       <c r="J121" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -5775,9 +5781,12 @@
       <c r="G122" s="11"/>
       <c r="H122" s="9"/>
       <c r="I122" s="15"/>
-      <c r="J122" s="7"/>
-    </row>
-    <row r="123" spans="1:10" ht="199.95" customHeight="1">
+      <c r="J122" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="199.9" customHeight="1">
       <c r="A123" s="48"/>
       <c r="B123" s="50" t="s">
         <v>252</v>
@@ -5804,7 +5813,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="199.95" customHeight="1">
+    <row r="124" spans="1:10" ht="199.9" customHeight="1">
       <c r="A124" s="48"/>
       <c r="B124" s="50"/>
       <c r="C124" s="49"/>
@@ -5830,7 +5839,7 @@
     <mergeCell ref="E123:E124"/>
     <mergeCell ref="F123:F124"/>
   </mergeCells>
-  <conditionalFormatting sqref="J1:J123 J125:J1048576">
+  <conditionalFormatting sqref="J125:J1048576 J1:J123">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>